<commit_message>
Clear paint colours and per-effect tile visuals; Smoldering debuff and Fortified tiles; comma-joined single letters; potion Use/Discard menu with tooltips; Effects glossary tab; cheaper trash (10 +5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qacman7MFobGSQncf5ZApG
</commit_message>
<xml_diff>
--- a/docs/art/Lexicore_UI_Act1_Buttons.xlsx
+++ b/docs/art/Lexicore_UI_Act1_Buttons.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buttons" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gameplay UI'!$A$1:$N$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gameplay UI'!$A$1:$N$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Background Act 1'!$A$1:$N$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Buttons'!$A$1:$N$10</definedName>
   </definedNames>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Lớp sơn tile (4 màu)</t>
+          <t>Tile sơn (4 màu)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Nền/vân sơn phủ lên tile: đỏ (Might), xanh dương (Robust), xanh lá (Agility), vàng (Fortune).</t>
+          <t>Cả mặt tile đổi màu sơn rõ ràng (không chỉ vân mờ): đỏ (Might), xanh dương (Robust), xanh lá (Agility), vàng (Fortune); vân sáp chéo + viền màu cùng tông, badge số cùng màu.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Lớp phủ trên tile + icon nhỏ: nhầy xanh chảy.</t>
+          <t>Lớp phủ trên tile + icon nhỏ: chất nhầy xanh chảy từ mép trên xuống.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Lớp phủ trên tile + icon nhỏ: giọt độc tím xanh.</t>
+          <t>Lớp phủ trên tile + icon nhỏ: tile ngả tím, giọt độc tím nhỏ xuống + bong bóng xanh.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Lớp phủ trên tile + icon nhỏ: ổ khoá.</t>
+          <t>Lớp phủ trên tile + icon nhỏ: tile xám tối, xích chéo + ổ khoá.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Lớp phủ trên tile + icon nhỏ: dấu X/đầu lâu.</t>
+          <t>Lớp phủ trên tile + icon nhỏ: dấu X đỏ to đè lên tile.</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Lớp phủ trên tile + icon nhỏ: con mắt nguyền tím.</t>
+          <t>Lớp phủ trên tile + icon nhỏ: hào quang tím đen + đầu lâu trắng ở góc.</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Lớp phủ trên tile + icon nhỏ: mây giận dữ/đám rối.</t>
+          <t>Lớp phủ trên tile + icon nhỏ: nét vẽ nguệch ngoạc cam + dấu giận đỏ.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2526,12 +2526,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ui_tile_fragile</t>
+          <t>ui_tile_deb_smoldering</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Overlay Fragile</t>
+          <t>Overlay debuff: smoldering</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Tile</t>
+          <t>Tile debuff</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Viền nét đứt + ngôi sao tím nhỏ góc trên phải (tile dùng 1 lần).</t>
+          <t>Lớp phủ trên tile + icon nhỏ: lửa cháy từ đáy tile + quầng sáng cam nhấp nháy (2 frame).</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -2586,12 +2586,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ui_tile_mini</t>
+          <t>ui_tile_fragile</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Tile mini</t>
+          <t>Overlay Fragile</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Claw machine; tooltip; deck list</t>
+          <t>Combat</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2621,18 +2621,18 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>80x80</t>
+          <t>176x176</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Phiên bản nhỏ của tile.</t>
+          <t>Vết nứt tím chằng chịt trên tile + viền nét đứt (tile dùng 1 lần là vỡ).</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2646,12 +2646,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ui_panel_paper</t>
+          <t>ui_tile_fortified</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Khung giấy kem</t>
+          <t>Overlay Fortified</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2661,17 +2661,17 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Tile</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Toàn game</t>
+          <t>Combat; Reward; Shop</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>9-slice</t>
+          <t>static</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2681,12 +2681,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>9-slice</t>
+          <t>176x176</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Hộp giấy kem viền mực đen mép run, bo góc lệch kiểu vẽ tay.</t>
+          <t>Tile bọc thép: mặt kim loại xám bóng, 4 đinh tán ở góc, vệt sáng chéo, viền đậm. Tile không bị discard và không dính debuff.</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -2706,12 +2706,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ui_modal</t>
+          <t>ui_tile_mini</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Popup / modal</t>
+          <t>Tile mini</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Tile</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Toàn game</t>
+          <t>Claw machine; tooltip; deck list</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>9-slice + nền tối mờ</t>
+          <t>static</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2741,18 +2741,18 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>9-slice</t>
+          <t>80x80</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Hộp popup trắng kem viền đen dày đổ bóng.</t>
+          <t>Phiên bản nhỏ của tile.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2766,12 +2766,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ui_tooltip</t>
+          <t>ui_panel_paper</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Tooltip</t>
+          <t>Khung giấy kem</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>9-slice + khung keyword phụ</t>
+          <t>9-slice</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Hộp tooltip tối/ kem kiểu Slay the Spire, có khung phụ giải thích keyword.</t>
+          <t>Hộp giấy kem viền mực đen mép run, bo góc lệch kiểu vẽ tay.</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -2826,12 +2826,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ui_toast</t>
+          <t>ui_modal</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Toast thông báo</t>
+          <t>Popup / modal</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2851,28 +2851,28 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
+          <t>9-slice + nền tối mờ</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
           <t>9-slice</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>9-slice</t>
-        </is>
-      </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Thanh đen bo góc chữ trắng ở dưới màn hình.</t>
+          <t>Hộp popup trắng kem viền đen dày đổ bóng.</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2886,12 +2886,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ui_hud_bar</t>
+          <t>ui_tooltip</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Thanh HUD (ngoài trận)</t>
+          <t>Tooltip</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2906,27 +2906,27 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Map; Shop; Rest; Events</t>
+          <t>Toàn game</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
+          <t>9-slice + khung keyword phụ</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
           <t>9-slice</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>3200x110</t>
-        </is>
-      </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Dải trắng viền đen chứa HP, gold, Act/Floor, potion, relic, nút Deck/Glossary/Achievements/Settings.</t>
+          <t>Hộp tooltip tối/ kem kiểu Slay the Spire, có khung phụ giải thích keyword.</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -2946,12 +2946,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ui_potion_slot</t>
+          <t>ui_toast</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Ô potion</t>
+          <t>Toast thông báo</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2966,33 +2966,33 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>HUD; Combat</t>
+          <t>Toàn game</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>filled; empty (viền đứt)</t>
+          <t>9-slice</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>88x88</t>
+          <t>9-slice</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Ô tròn/vuông nhỏ chứa lọ potion.</t>
+          <t>Thanh đen bo góc chữ trắng ở dưới màn hình.</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3006,32 +3006,32 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>icon_hud_gold</t>
+          <t>ui_hud_bar</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Icon gold</t>
+          <t>Thanh HUD (ngoài trận)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>HUD</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Combat (bảng góc phải); HUD</t>
+          <t>Map; Shop; Rest; Events</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>static</t>
+          <t>9-slice</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -3041,12 +3041,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>120x120</t>
+          <t>3200x110</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Icon lớn vẽ sáp: túi vàng.</t>
+          <t>Dải trắng viền đen chứa HP, gold, Act/Floor, potion, relic, nút Deck/Glossary/Achievements/Settings.</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -3066,47 +3066,47 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>icon_hud_map</t>
+          <t>ui_potion_slot</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Icon map</t>
+          <t>Ô potion</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>HUD</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Combat (bảng góc phải); HUD</t>
+          <t>HUD; Combat</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>static</t>
+          <t>filled; empty (viền đứt)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>120x120</t>
+          <t>88x88</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Icon lớn vẽ sáp: bản đồ.</t>
+          <t>Ô tròn/vuông nhỏ chứa lọ potion.</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -3126,12 +3126,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>icon_hud_deck</t>
+          <t>icon_hud_gold</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Icon deck</t>
+          <t>Icon gold</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Icon lớn vẽ sáp: xấp tile.</t>
+          <t>Icon lớn vẽ sáp: túi vàng.</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -3186,12 +3186,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>icon_hud_gear</t>
+          <t>icon_hud_map</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Icon gear</t>
+          <t>Icon map</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Icon lớn vẽ sáp: bánh răng (Settings).</t>
+          <t>Icon lớn vẽ sáp: bản đồ.</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -3246,12 +3246,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>icon_heart</t>
+          <t>icon_hud_deck</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Icon nhỏ heart</t>
+          <t>Icon deck</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>HUD</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>HUD; intent; text</t>
+          <t>Combat (bảng góc phải); HUD</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3281,12 +3281,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>48x48</t>
+          <t>120x120</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>trái tim đỏ (HP)</t>
+          <t>Icon lớn vẽ sáp: xấp tile.</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
@@ -3306,12 +3306,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>icon_coin</t>
+          <t>icon_hud_gear</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Icon nhỏ coin</t>
+          <t>Icon gear</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3321,12 +3321,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>HUD</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>HUD; intent; text</t>
+          <t>Combat (bảng góc phải); HUD</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3341,12 +3341,12 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>48x48</t>
+          <t>120x120</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>đồng xu vàng (gold)</t>
+          <t>Icon lớn vẽ sáp: bánh răng (Settings).</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -3366,12 +3366,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>icon_atk</t>
+          <t>icon_heart</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Icon nhỏ atk</t>
+          <t>Icon nhỏ heart</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>kiếm (intent tấn công)</t>
+          <t>trái tim đỏ (HP)</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
@@ -3426,12 +3426,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>icon_blk</t>
+          <t>icon_coin</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Icon nhỏ blk</t>
+          <t>Icon nhỏ coin</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>khiên xanh (intent block)</t>
+          <t>đồng xu vàng (gold)</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
@@ -3486,12 +3486,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>icon_buff</t>
+          <t>icon_atk</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Icon nhỏ buff</t>
+          <t>Icon nhỏ atk</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>mũi tên đỏ đi lên (buff)</t>
+          <t>kiếm (intent tấn công)</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
@@ -3546,12 +3546,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>icon_skill</t>
+          <t>icon_blk</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Icon nhỏ skill</t>
+          <t>Icon nhỏ blk</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>ngôi sao tím (kỹ năng)</t>
+          <t>khiên xanh (intent block)</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
@@ -3606,12 +3606,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>icon_status_block</t>
+          <t>icon_buff</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Status: block</t>
+          <t>Icon nhỏ buff</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3621,12 +3621,12 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Status/Intent</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Combat; Tooltip; Glossary</t>
+          <t>HUD; intent; text</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3641,12 +3641,12 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>64x64</t>
+          <t>48x48</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>khiên xanh</t>
+          <t>mũi tên đỏ đi lên (buff)</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
@@ -3666,12 +3666,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>icon_status_might</t>
+          <t>icon_skill</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Status: might</t>
+          <t>Icon nhỏ skill</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3681,12 +3681,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Status/Intent</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Combat; Tooltip; Glossary</t>
+          <t>HUD; intent; text</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3701,12 +3701,12 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>64x64</t>
+          <t>48x48</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>nắm đấm/mũi tên đỏ</t>
+          <t>ngôi sao tím (kỹ năng)</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
@@ -3726,12 +3726,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>icon_status_robust</t>
+          <t>icon_status_block</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Status: robust</t>
+          <t>Status: block</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>khiên xanh nhạt có dấu +</t>
+          <t>khiên xanh</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
@@ -3786,12 +3786,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>icon_status_thorns</t>
+          <t>icon_status_might</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Status: thorns</t>
+          <t>Status: might</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>gai</t>
+          <t>nắm đấm/mũi tên đỏ</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
@@ -3846,12 +3846,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>icon_status_poison</t>
+          <t>icon_status_robust</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Status: poison</t>
+          <t>Status: robust</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>giọt độc xanh</t>
+          <t>khiên xanh nhạt có dấu +</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
@@ -3906,12 +3906,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>icon_status_weaken</t>
+          <t>icon_status_thorns</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Status: weaken</t>
+          <t>Status: thorns</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>khiên nứt</t>
+          <t>gai</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
@@ -3966,12 +3966,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>icon_status_broken</t>
+          <t>icon_status_poison</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Status: broken</t>
+          <t>Status: poison</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>trái tim/khiên vỡ</t>
+          <t>giọt độc xanh</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
@@ -4026,12 +4026,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>icon_status_curse</t>
+          <t>icon_status_weaken</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Status: curse</t>
+          <t>Status: weaken</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>con mắt nguyền tím</t>
+          <t>khiên nứt</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
@@ -4086,12 +4086,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>icon_status_frustrated</t>
+          <t>icon_status_broken</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Status: frustrated</t>
+          <t>Status: broken</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>mây giận</t>
+          <t>trái tim/khiên vỡ</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
@@ -4146,12 +4146,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>icon_status_slimy</t>
+          <t>icon_status_curse</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Status: slimy</t>
+          <t>Status: curse</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>giọt nhầy</t>
+          <t>con mắt nguyền tím</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
@@ -4206,12 +4206,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>icon_status_lock</t>
+          <t>icon_status_frustrated</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Status: lock</t>
+          <t>Status: frustrated</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>ổ khoá</t>
+          <t>mây giận</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
@@ -4266,12 +4266,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>icon_status_condemn</t>
+          <t>icon_status_slimy</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Status: condemn</t>
+          <t>Status: slimy</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>đầu lâu/X</t>
+          <t>giọt nhầy</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
@@ -4326,12 +4326,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>icon_status_energy</t>
+          <t>icon_status_lock</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Status: energy</t>
+          <t>Status: lock</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>tia sét/ngọc energy</t>
+          <t>ổ khoá</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
@@ -4386,12 +4386,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>icon_status_crit</t>
+          <t>icon_status_condemn</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Status: crit</t>
+          <t>Status: condemn</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>tia sáng crit</t>
+          <t>đầu lâu/X</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
@@ -4446,12 +4446,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>icon_status_intentAtk</t>
+          <t>icon_status_energy</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Status: intentAtk</t>
+          <t>Status: energy</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>kiếm (intent đánh)</t>
+          <t>tia sét/ngọc energy</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
@@ -4506,12 +4506,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>icon_status_intentBlk</t>
+          <t>icon_status_crit</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Status: intentBlk</t>
+          <t>Status: crit</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>khiên (intent thủ)</t>
+          <t>tia sáng crit</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
@@ -4566,12 +4566,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>icon_status_intentBuff</t>
+          <t>icon_status_intentAtk</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Status: intentBuff</t>
+          <t>Status: intentAtk</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>mũi tên lên (intent buff)</t>
+          <t>kiếm (intent đánh)</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
@@ -4626,12 +4626,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>icon_status_intentDebuff</t>
+          <t>icon_status_intentBlk</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Status: intentDebuff</t>
+          <t>Status: intentBlk</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>vòng xoáy tím (intent debuff)</t>
+          <t>khiên (intent thủ)</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
@@ -4686,12 +4686,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>icon_status_intentTile</t>
+          <t>icon_status_intentBuff</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Status: intentTile</t>
+          <t>Status: intentBuff</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>tile có vết bẩn (intent gây debuff tile)</t>
+          <t>mũi tên lên (intent buff)</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
@@ -4746,12 +4746,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>icon_status_intentSummon</t>
+          <t>icon_status_intentDebuff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Status: intentSummon</t>
+          <t>Status: intentDebuff</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>nấm con có dấu + (intent triệu hồi)</t>
+          <t>vòng xoáy tím (intent debuff)</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
@@ -4803,8 +4803,308 @@
       <c r="M72" s="2" t="inlineStr"/>
       <c r="N72" s="2" t="inlineStr"/>
     </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>icon_status_intentTile</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Status: intentTile</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Status/Intent</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Combat; Tooltip; Glossary</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>64x64</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>tile có vết bẩn (intent gây debuff tile)</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr"/>
+      <c r="N73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>icon_status_intentSummon</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Status: intentSummon</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Status/Intent</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Combat; Tooltip; Glossary</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>64x64</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>nấm con có dấu + (intent triệu hồi)</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr"/>
+      <c r="N74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>icon_status_burn</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Status: burn</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Status/Intent</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Combat; Tooltip; Glossary</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>64x64</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>ngọn lửa cam (Smoldering)</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr"/>
+      <c r="N75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>icon_status_fortified</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Status: fortified</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Status/Intent</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Combat; Tooltip; Glossary</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>64x64</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>khiên thép có đinh tán (Fortified)</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>icon_status_fragile</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Status: fragile</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Status/Intent</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Combat; Tooltip; Glossary</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>64x64</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>ô vuông nứt tím (Fragile)</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N72"/>
+  <autoFilter ref="A1:N77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>